<commit_message>
Sept 19 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/T2018_GiftLog_GiftApprovalProcess_ApproveGifts_VerifyThePreviousYTDGiftValueAndNewYTDIsVisibleToApprover.xlsx
+++ b/TestData/T2018_GiftLog_GiftApprovalProcess_ApproveGifts_VerifyThePreviousYTDGiftValueAndNewYTDIsVisibleToApprover.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\HL\SalesForce_Project\SalesForce_Project\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{278CDD53-C0AF-4450-A15A-BB5A0637BA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F88C1CB-4D2B-49DC-8791-5D5559D4F287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="GiftLog" sheetId="4" r:id="rId1"/>
-    <sheet name="GiftEdit" sheetId="6" r:id="rId2"/>
-    <sheet name="Users" sheetId="5" r:id="rId3"/>
+    <sheet name="Users" sheetId="5" r:id="rId1"/>
+    <sheet name="AppName" sheetId="7" r:id="rId2"/>
+    <sheet name="ModuleName" sheetId="8" r:id="rId3"/>
+    <sheet name="GiftLog" sheetId="4" r:id="rId4"/>
+    <sheet name="GiftEdit" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
   <si>
     <t>Client Gift Pre-approval</t>
   </si>
@@ -128,9 +130,6 @@
     <t>ComplianceUser</t>
   </si>
   <si>
-    <t>Julie Carthane</t>
-  </si>
-  <si>
     <t>Australian Dollar</t>
   </si>
   <si>
@@ -144,6 +143,21 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>Melissa Zatta</t>
+  </si>
+  <si>
+    <t>Zain Sheikh</t>
+  </si>
+  <si>
+    <t>App Name</t>
+  </si>
+  <si>
+    <t>HL Banker</t>
+  </si>
+  <si>
+    <t>Gift Requests</t>
   </si>
 </sst>
 </file>
@@ -187,11 +201,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -473,104 +490,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.109375" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="B2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" t="s">
-        <v>31</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2" t="s">
-        <v>20</v>
-      </c>
-      <c r="M2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -580,69 +521,144 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F9CF030-9264-47AF-8ECE-ED5E390216BF}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F411CF1E-2426-42DB-8C45-A4CB0B21CB33}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>34</v>
+        <v>30</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E2" t="s">
-        <v>27</v>
-      </c>
-      <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" t="s">
         <v>35</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H2" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -651,29 +667,70 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
         <v>33</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>